<commit_message>
Split TinyTMR into 2 parts.
</commit_message>
<xml_diff>
--- a/FrontendTMR/Fabrication/BOM_TinyTMR.xlsx
+++ b/FrontendTMR/Fabrication/BOM_TinyTMR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TinyTMR\FrontendTMR\Fabrication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A2180E4-02E6-4C19-B311-225CCA3C2ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C78FE1E-BBCE-4439-913E-6C40E634753D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28830" windowHeight="14115" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="psu" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="357">
   <si>
     <t>Item</t>
   </si>
@@ -1591,12 +1590,42 @@
   <si>
     <t>R1,R2,R6,R7,R9,R12,R18,R21,R30,R34,R62,R67,R75</t>
   </si>
+  <si>
+    <t>J3,J5</t>
+  </si>
+  <si>
+    <t>J4,J6</t>
+  </si>
+  <si>
+    <t>CONN-2x2P-Male</t>
+  </si>
+  <si>
+    <t>CONN-2x2P-Female</t>
+  </si>
+  <si>
+    <t>HCTL(华灿天禄)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    PZ200-2-02-W-2.0-G1</t>
+  </si>
+  <si>
+    <t>CONN-2X2P_2D0_DEG90</t>
+  </si>
+  <si>
+    <t>C19270583</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    PM200-2-02-W-4.3</t>
+  </si>
+  <si>
+    <t>C3012185</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1761,6 +1790,13 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="1"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -2104,8 +2140,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - 着色 1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2340,18 +2379,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="3" max="3" width="36" customWidth="1"/>
     <col min="4" max="4" width="17.875" customWidth="1"/>
-    <col min="5" max="5" width="18.25" customWidth="1"/>
+    <col min="5" max="5" width="24.25" customWidth="1"/>
     <col min="6" max="6" width="14.625" customWidth="1"/>
     <col min="7" max="7" width="19.5" customWidth="1"/>
     <col min="8" max="8" width="26.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75">
+    <row r="1" spans="1:8" ht="26.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2367,7 +2406,7 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
@@ -3032,25 +3071,25 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>347</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>349</v>
       </c>
       <c r="E27" t="s">
-        <v>123</v>
+        <v>353</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>354</v>
       </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>351</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
+        <v>352</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -3058,25 +3097,25 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>126</v>
+        <v>348</v>
       </c>
       <c r="D28" t="s">
-        <v>127</v>
+        <v>350</v>
       </c>
       <c r="E28" t="s">
-        <v>128</v>
+        <v>353</v>
       </c>
       <c r="F28" t="s">
-        <v>129</v>
+        <v>356</v>
       </c>
       <c r="G28" t="s">
-        <v>12</v>
+        <v>351</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>355</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3084,25 +3123,25 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D29" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E29" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="G29" t="s">
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3113,22 +3152,22 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E30" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="F30" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G30" t="s">
         <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -3136,25 +3175,25 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="D31" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E31" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F31" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="G31" t="s">
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3165,22 +3204,22 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D32" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="E32" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="F32" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="G32" t="s">
-        <v>150</v>
+        <v>12</v>
       </c>
       <c r="H32" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3191,22 +3230,22 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="D33" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="E33" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="F33" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="G33" t="s">
-        <v>155</v>
+        <v>12</v>
       </c>
       <c r="H33" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3217,22 +3256,22 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="D34" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="E34" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F34" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G34" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="H34" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -3240,25 +3279,25 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>346</v>
+        <v>151</v>
       </c>
       <c r="D35" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="E35" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="F35" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="G35" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="H35" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -3266,25 +3305,25 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="E36" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="F36" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="G36" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="H36" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -3292,25 +3331,25 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C37" t="s">
-        <v>170</v>
+        <v>346</v>
       </c>
       <c r="D37" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="E37" t="s">
         <v>162</v>
       </c>
       <c r="F37" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="G37" t="s">
         <v>164</v>
       </c>
       <c r="H37" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -3321,22 +3360,22 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D38" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="E38" t="s">
         <v>162</v>
       </c>
       <c r="F38" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="G38" t="s">
         <v>164</v>
       </c>
       <c r="H38" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3344,25 +3383,25 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D39" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="E39" t="s">
         <v>162</v>
       </c>
       <c r="F39" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="G39" t="s">
         <v>164</v>
       </c>
       <c r="H39" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3370,25 +3409,25 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D40" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="E40" t="s">
         <v>162</v>
       </c>
       <c r="F40" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G40" t="s">
         <v>164</v>
       </c>
       <c r="H40" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -3399,22 +3438,22 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D41" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="E41" t="s">
         <v>162</v>
       </c>
       <c r="F41" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="G41" t="s">
         <v>164</v>
       </c>
       <c r="H41" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3422,25 +3461,25 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D42" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="E42" t="s">
         <v>162</v>
       </c>
       <c r="F42" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="G42" t="s">
         <v>164</v>
       </c>
       <c r="H42" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -3451,22 +3490,22 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D43" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="E43" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F43" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="G43" t="s">
         <v>164</v>
       </c>
       <c r="H43" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -3474,25 +3513,25 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D44" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="E44" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F44" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G44" t="s">
         <v>164</v>
       </c>
       <c r="H44" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -3503,22 +3542,22 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D45" t="s">
-        <v>203</v>
+        <v>161</v>
       </c>
       <c r="E45" t="s">
         <v>195</v>
       </c>
       <c r="F45" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="G45" t="s">
         <v>164</v>
       </c>
       <c r="H45" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -3526,25 +3565,25 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D46" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E46" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="F46" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="G46" t="s">
         <v>164</v>
       </c>
       <c r="H46" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -3552,25 +3591,25 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D47" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="E47" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="F47" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="G47" t="s">
         <v>164</v>
       </c>
       <c r="H47" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -3578,25 +3617,25 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C48" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="D48" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="E48" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F48" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G48" t="s">
         <v>164</v>
       </c>
       <c r="H48" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -3604,25 +3643,25 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="D49" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="E49" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F49" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="G49" t="s">
         <v>164</v>
       </c>
       <c r="H49" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -3630,25 +3669,25 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D50" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E50" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="F50" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="G50" t="s">
         <v>164</v>
       </c>
       <c r="H50" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -3656,25 +3695,25 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C51" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="D51" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
       <c r="E51" t="s">
         <v>195</v>
       </c>
       <c r="F51" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="G51" t="s">
         <v>164</v>
       </c>
       <c r="H51" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -3682,25 +3721,25 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D52" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="E52" t="s">
         <v>162</v>
       </c>
       <c r="F52" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="G52" t="s">
         <v>164</v>
       </c>
       <c r="H52" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -3708,25 +3747,25 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C53" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D53" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="E53" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="F53" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="G53" t="s">
         <v>164</v>
       </c>
       <c r="H53" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -3734,25 +3773,25 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="D54" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="E54" t="s">
         <v>162</v>
       </c>
       <c r="F54" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="G54" t="s">
         <v>164</v>
       </c>
       <c r="H54" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -3760,25 +3799,25 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D55" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E55" t="s">
         <v>162</v>
       </c>
       <c r="F55" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G55" t="s">
         <v>164</v>
       </c>
       <c r="H55" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -3789,22 +3828,22 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="D56" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="E56" t="s">
         <v>162</v>
       </c>
       <c r="F56" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="G56" t="s">
         <v>164</v>
       </c>
       <c r="H56" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -3812,25 +3851,25 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="D57" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E57" t="s">
         <v>162</v>
       </c>
       <c r="F57" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G57" t="s">
         <v>164</v>
       </c>
       <c r="H57" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -3841,22 +3880,22 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="D58" t="s">
-        <v>203</v>
+        <v>246</v>
       </c>
       <c r="E58" t="s">
         <v>162</v>
       </c>
       <c r="F58" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="G58" t="s">
         <v>164</v>
       </c>
       <c r="H58" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -3867,22 +3906,22 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D59" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="E59" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F59" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="G59" t="s">
         <v>164</v>
       </c>
       <c r="H59" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -3893,22 +3932,22 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D60" t="s">
-        <v>261</v>
+        <v>203</v>
       </c>
       <c r="E60" t="s">
         <v>162</v>
       </c>
       <c r="F60" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="G60" t="s">
         <v>164</v>
       </c>
       <c r="H60" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -3919,22 +3958,22 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D61" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="E61" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="F61" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="G61" t="s">
         <v>164</v>
       </c>
       <c r="H61" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -3945,22 +3984,22 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="D62" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="E62" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="F62" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="G62" t="s">
         <v>164</v>
       </c>
       <c r="H62" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -3971,22 +4010,22 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="D63" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="E63" t="s">
         <v>162</v>
       </c>
       <c r="F63" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="G63" t="s">
         <v>164</v>
       </c>
       <c r="H63" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -3994,25 +4033,25 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="D64" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="E64" t="s">
-        <v>278</v>
+        <v>195</v>
       </c>
       <c r="F64" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="G64" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="H64" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -4023,22 +4062,22 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="D65" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="E65" t="s">
-        <v>282</v>
+        <v>162</v>
       </c>
       <c r="F65" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="G65" t="s">
-        <v>284</v>
+        <v>164</v>
       </c>
       <c r="H65" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -4046,25 +4085,25 @@
         <v>65</v>
       </c>
       <c r="B66">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C66" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D66" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="E66" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F66" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="G66" t="s">
-        <v>284</v>
+        <v>12</v>
       </c>
       <c r="H66" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -4075,22 +4114,22 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="D67" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="E67" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="F67" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="G67" t="s">
         <v>284</v>
       </c>
       <c r="H67" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -4101,22 +4140,22 @@
         <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="D68" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="E68" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F68" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="G68" t="s">
         <v>284</v>
       </c>
       <c r="H68" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -4127,22 +4166,22 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D69" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="E69" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="F69" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="G69" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="H69" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -4153,19 +4192,22 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="D70" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="E70" t="s">
-        <v>304</v>
+        <v>291</v>
+      </c>
+      <c r="F70" t="s">
+        <v>295</v>
       </c>
       <c r="G70" t="s">
-        <v>305</v>
+        <v>284</v>
       </c>
       <c r="H70" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -4173,25 +4215,25 @@
         <v>70</v>
       </c>
       <c r="B71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="D71" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="E71" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="F71" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="G71" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="H71" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -4202,22 +4244,19 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="D72" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="E72" t="s">
-        <v>313</v>
-      </c>
-      <c r="F72" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="G72" t="s">
-        <v>284</v>
+        <v>305</v>
       </c>
       <c r="H72" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -4225,25 +4264,25 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="D73" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="E73" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="F73" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="G73" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="H73" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -4254,22 +4293,22 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="D74" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="E74" t="s">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="F74" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="G74" t="s">
-        <v>99</v>
+        <v>284</v>
       </c>
       <c r="H74" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -4280,22 +4319,22 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="D75" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="E75" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="F75" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="G75" t="s">
-        <v>328</v>
+        <v>300</v>
       </c>
       <c r="H75" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -4306,22 +4345,22 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="D76" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="E76" t="s">
-        <v>332</v>
+        <v>287</v>
       </c>
       <c r="F76" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="G76" t="s">
-        <v>334</v>
+        <v>99</v>
       </c>
       <c r="H76" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -4332,22 +4371,22 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="D77" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="E77" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="F77" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="G77" t="s">
-        <v>284</v>
+        <v>328</v>
       </c>
       <c r="H77" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -4358,26 +4397,78 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
+        <v>330</v>
+      </c>
+      <c r="D78" t="s">
+        <v>331</v>
+      </c>
+      <c r="E78" t="s">
+        <v>332</v>
+      </c>
+      <c r="F78" t="s">
+        <v>333</v>
+      </c>
+      <c r="G78" t="s">
+        <v>334</v>
+      </c>
+      <c r="H78" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>335</v>
+      </c>
+      <c r="D79" t="s">
+        <v>336</v>
+      </c>
+      <c r="E79" t="s">
+        <v>337</v>
+      </c>
+      <c r="F79" t="s">
+        <v>338</v>
+      </c>
+      <c r="G79" t="s">
+        <v>284</v>
+      </c>
+      <c r="H79" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
         <v>340</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D80" t="s">
         <v>341</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E80" t="s">
         <v>342</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F80" t="s">
         <v>343</v>
       </c>
-      <c r="G78" t="s">
+      <c r="G80" t="s">
         <v>344</v>
       </c>
-      <c r="H78" t="s">
+      <c r="H80" t="s">
         <v>345</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>